<commit_message>
Sincronizaci├│n autom├ítica 13/02/2026 16:27:27.54
</commit_message>
<xml_diff>
--- a/Fichas/O956.xlsx
+++ b/Fichas/O956.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\DESKTOP-ID9UEKK\Users\Admin\Desktop\CONTROL DISEÑO\VIVA ROUSS\OPTIMA\O956 TOP BANDITA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBCAA2B1-6303-4C87-853B-DD6550BAD7C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F1676AE-B328-4DE8-8DB2-D9CD41715932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="38">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -808,100 +808,130 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="5" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="14" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -910,10 +940,112 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="46" fontId="12" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="46" fontId="12" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="45" fontId="19" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="19" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="19" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="19" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="7" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="7" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="19" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="19" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="19" fillId="13" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="19" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="7" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="7" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -946,6 +1078,108 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -964,285 +1198,6 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="14" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="19" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="19" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="19" fillId="13" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="19" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="46" fontId="7" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="46" fontId="7" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="18" fillId="12" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="18" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="18" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="18" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="19" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="19" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="19" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="45" fontId="19" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="46" fontId="7" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="46" fontId="7" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1268,27 +1223,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1303,13 +1237,100 @@
     <xf numFmtId="0" fontId="28" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="18" fillId="12" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="18" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="18" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="18" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="12" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="12" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1330,6 +1351,9 @@
     <xf numFmtId="0" fontId="17" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1337,30 +1361,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="5" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1791,622 +1791,618 @@
       <c r="O1" s="1"/>
     </row>
     <row r="2" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="46" t="s">
+      <c r="C2" s="87"/>
+      <c r="D2" s="87"/>
+      <c r="E2" s="90" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-      <c r="L2" s="47"/>
-      <c r="M2" s="47"/>
-      <c r="N2" s="47"/>
-      <c r="O2" s="48"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
+      <c r="H2" s="91"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="91"/>
+      <c r="K2" s="91"/>
+      <c r="L2" s="91"/>
+      <c r="M2" s="91"/>
+      <c r="N2" s="91"/>
+      <c r="O2" s="92"/>
     </row>
     <row r="3" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="44"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="50"/>
-      <c r="I3" s="50"/>
-      <c r="J3" s="50"/>
-      <c r="K3" s="50"/>
-      <c r="L3" s="50"/>
-      <c r="M3" s="50"/>
-      <c r="N3" s="50"/>
-      <c r="O3" s="51"/>
+      <c r="B3" s="88"/>
+      <c r="C3" s="89"/>
+      <c r="D3" s="89"/>
+      <c r="E3" s="93"/>
+      <c r="F3" s="94"/>
+      <c r="G3" s="94"/>
+      <c r="H3" s="94"/>
+      <c r="I3" s="94"/>
+      <c r="J3" s="94"/>
+      <c r="K3" s="94"/>
+      <c r="L3" s="94"/>
+      <c r="M3" s="94"/>
+      <c r="N3" s="94"/>
+      <c r="O3" s="95"/>
     </row>
     <row r="4" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
-      <c r="E4" s="52" t="s">
+      <c r="E4" s="130" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="53"/>
-      <c r="G4" s="53"/>
-      <c r="H4" s="53"/>
-      <c r="I4" s="53"/>
-      <c r="J4" s="53"/>
-      <c r="K4" s="53"/>
-      <c r="L4" s="53"/>
-      <c r="M4" s="53"/>
-      <c r="N4" s="53"/>
-      <c r="O4" s="54"/>
+      <c r="F4" s="131"/>
+      <c r="G4" s="131"/>
+      <c r="H4" s="131"/>
+      <c r="I4" s="131"/>
+      <c r="J4" s="131"/>
+      <c r="K4" s="131"/>
+      <c r="L4" s="131"/>
+      <c r="M4" s="131"/>
+      <c r="N4" s="131"/>
+      <c r="O4" s="132"/>
     </row>
     <row r="5" spans="1:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="55"/>
-      <c r="F5" s="56"/>
-      <c r="G5" s="56"/>
-      <c r="H5" s="56"/>
-      <c r="I5" s="56"/>
-      <c r="J5" s="56"/>
-      <c r="K5" s="56"/>
-      <c r="L5" s="56"/>
-      <c r="M5" s="56"/>
-      <c r="N5" s="56"/>
-      <c r="O5" s="57"/>
+      <c r="E5" s="133"/>
+      <c r="F5" s="134"/>
+      <c r="G5" s="134"/>
+      <c r="H5" s="134"/>
+      <c r="I5" s="134"/>
+      <c r="J5" s="134"/>
+      <c r="K5" s="134"/>
+      <c r="L5" s="134"/>
+      <c r="M5" s="134"/>
+      <c r="N5" s="134"/>
+      <c r="O5" s="135"/>
     </row>
     <row r="6" spans="1:15" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="2"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
-      <c r="E6" s="151"/>
-      <c r="F6" s="152"/>
-      <c r="G6" s="152"/>
-      <c r="H6" s="152"/>
-      <c r="I6" s="152"/>
-      <c r="J6" s="152"/>
-      <c r="K6" s="152"/>
-      <c r="L6" s="152"/>
-      <c r="M6" s="152"/>
-      <c r="N6" s="152"/>
-      <c r="O6" s="153"/>
+      <c r="E6" s="136"/>
+      <c r="F6" s="137"/>
+      <c r="G6" s="137"/>
+      <c r="H6" s="137"/>
+      <c r="I6" s="137"/>
+      <c r="J6" s="137"/>
+      <c r="K6" s="137"/>
+      <c r="L6" s="137"/>
+      <c r="M6" s="137"/>
+      <c r="N6" s="137"/>
+      <c r="O6" s="138"/>
     </row>
     <row r="7" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
-      <c r="E7" s="38" t="s">
+      <c r="E7" s="48" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="39"/>
-      <c r="G7" s="104" t="s">
+      <c r="F7" s="49"/>
+      <c r="G7" s="96" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="105"/>
-      <c r="I7" s="106"/>
-      <c r="J7" s="75" t="s">
+      <c r="H7" s="97"/>
+      <c r="I7" s="98"/>
+      <c r="J7" s="102" t="s">
         <v>32</v>
       </c>
-      <c r="K7" s="76"/>
-      <c r="L7" s="77"/>
-      <c r="M7" s="93"/>
-      <c r="N7" s="93"/>
-      <c r="O7" s="94"/>
+      <c r="K7" s="103"/>
+      <c r="L7" s="104"/>
+      <c r="M7" s="108"/>
+      <c r="N7" s="108"/>
+      <c r="O7" s="109"/>
     </row>
     <row r="8" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="107"/>
-      <c r="H8" s="108"/>
-      <c r="I8" s="109"/>
-      <c r="J8" s="78"/>
-      <c r="K8" s="79"/>
-      <c r="L8" s="80"/>
-      <c r="M8" s="95"/>
-      <c r="N8" s="95"/>
-      <c r="O8" s="96"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="49"/>
+      <c r="G8" s="99"/>
+      <c r="H8" s="100"/>
+      <c r="I8" s="101"/>
+      <c r="J8" s="105"/>
+      <c r="K8" s="106"/>
+      <c r="L8" s="107"/>
+      <c r="M8" s="110"/>
+      <c r="N8" s="110"/>
+      <c r="O8" s="111"/>
     </row>
     <row r="9" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="2"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
-      <c r="E9" s="38" t="s">
+      <c r="E9" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="F9" s="39"/>
-      <c r="G9" s="154" t="s">
+      <c r="F9" s="49"/>
+      <c r="G9" s="139" t="s">
         <v>28</v>
       </c>
-      <c r="H9" s="155"/>
-      <c r="I9" s="155"/>
-      <c r="J9" s="155"/>
-      <c r="K9" s="155"/>
-      <c r="L9" s="155"/>
-      <c r="M9" s="155"/>
-      <c r="N9" s="155"/>
-      <c r="O9" s="156"/>
+      <c r="H9" s="140"/>
+      <c r="I9" s="140"/>
+      <c r="J9" s="140"/>
+      <c r="K9" s="140"/>
+      <c r="L9" s="140"/>
+      <c r="M9" s="140"/>
+      <c r="N9" s="140"/>
+      <c r="O9" s="141"/>
     </row>
     <row r="10" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="2"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="157"/>
-      <c r="H10" s="158"/>
-      <c r="I10" s="158"/>
-      <c r="J10" s="158"/>
-      <c r="K10" s="158"/>
-      <c r="L10" s="158"/>
-      <c r="M10" s="158"/>
-      <c r="N10" s="158"/>
-      <c r="O10" s="159"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="142"/>
+      <c r="H10" s="143"/>
+      <c r="I10" s="143"/>
+      <c r="J10" s="143"/>
+      <c r="K10" s="143"/>
+      <c r="L10" s="143"/>
+      <c r="M10" s="143"/>
+      <c r="N10" s="143"/>
+      <c r="O10" s="144"/>
     </row>
     <row r="11" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
-      <c r="E11" s="38" t="s">
+      <c r="E11" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="F11" s="39"/>
-      <c r="G11" s="160" t="s">
+      <c r="F11" s="49"/>
+      <c r="G11" s="112" t="s">
         <v>33</v>
       </c>
-      <c r="H11" s="110"/>
-      <c r="I11" s="111"/>
-      <c r="J11" s="161" t="s">
+      <c r="H11" s="113"/>
+      <c r="I11" s="114"/>
+      <c r="J11" s="118" t="s">
         <v>34</v>
       </c>
-      <c r="K11" s="162"/>
-      <c r="L11" s="163"/>
-      <c r="M11" s="115"/>
-      <c r="N11" s="116"/>
-      <c r="O11" s="117"/>
+      <c r="K11" s="119"/>
+      <c r="L11" s="120"/>
+      <c r="M11" s="124"/>
+      <c r="N11" s="125"/>
+      <c r="O11" s="126"/>
     </row>
     <row r="12" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="2"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="112"/>
-      <c r="H12" s="113"/>
-      <c r="I12" s="114"/>
-      <c r="J12" s="164"/>
-      <c r="K12" s="165"/>
-      <c r="L12" s="166"/>
-      <c r="M12" s="118"/>
-      <c r="N12" s="119"/>
-      <c r="O12" s="120"/>
+      <c r="E12" s="48"/>
+      <c r="F12" s="49"/>
+      <c r="G12" s="115"/>
+      <c r="H12" s="116"/>
+      <c r="I12" s="117"/>
+      <c r="J12" s="121"/>
+      <c r="K12" s="122"/>
+      <c r="L12" s="123"/>
+      <c r="M12" s="127"/>
+      <c r="N12" s="128"/>
+      <c r="O12" s="129"/>
     </row>
     <row r="13" spans="1:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="2"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
-      <c r="E13" s="167" t="s">
+      <c r="E13" s="145" t="s">
         <v>24</v>
       </c>
-      <c r="F13" s="168"/>
-      <c r="G13" s="121">
+      <c r="F13" s="146"/>
+      <c r="G13" s="149">
         <f>80*110%</f>
         <v>88</v>
       </c>
-      <c r="H13" s="122"/>
-      <c r="I13" s="125" t="s">
+      <c r="H13" s="150"/>
+      <c r="I13" s="153" t="s">
         <v>6</v>
       </c>
-      <c r="J13" s="87">
+      <c r="J13" s="155">
         <f>93*110%</f>
         <v>102.30000000000001</v>
       </c>
-      <c r="K13" s="88"/>
-      <c r="L13" s="91" t="s">
+      <c r="K13" s="156"/>
+      <c r="L13" s="159" t="s">
         <v>6</v>
       </c>
-      <c r="M13" s="127"/>
-      <c r="N13" s="34"/>
-      <c r="O13" s="36"/>
+      <c r="M13" s="161"/>
+      <c r="N13" s="162"/>
+      <c r="O13" s="165"/>
     </row>
     <row r="14" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
-      <c r="E14" s="169"/>
-      <c r="F14" s="170"/>
-      <c r="G14" s="123"/>
-      <c r="H14" s="124"/>
-      <c r="I14" s="126"/>
-      <c r="J14" s="89"/>
-      <c r="K14" s="90"/>
-      <c r="L14" s="92"/>
-      <c r="M14" s="128"/>
-      <c r="N14" s="35"/>
-      <c r="O14" s="37"/>
+      <c r="E14" s="147"/>
+      <c r="F14" s="148"/>
+      <c r="G14" s="151"/>
+      <c r="H14" s="152"/>
+      <c r="I14" s="154"/>
+      <c r="J14" s="157"/>
+      <c r="K14" s="158"/>
+      <c r="L14" s="160"/>
+      <c r="M14" s="163"/>
+      <c r="N14" s="164"/>
+      <c r="O14" s="166"/>
     </row>
     <row r="15" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="2"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
-      <c r="E15" s="38" t="s">
+      <c r="E15" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="F15" s="39"/>
-      <c r="G15" s="134">
+      <c r="F15" s="49"/>
+      <c r="G15" s="50">
         <v>3.2407407407407406E-3</v>
       </c>
-      <c r="H15" s="135"/>
-      <c r="I15" s="138" t="s">
+      <c r="H15" s="51"/>
+      <c r="I15" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="J15" s="81">
+      <c r="J15" s="56">
         <v>1.9675925925925924E-3</v>
       </c>
-      <c r="K15" s="82"/>
-      <c r="L15" s="85" t="s">
+      <c r="K15" s="57"/>
+      <c r="L15" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="M15" s="129"/>
-      <c r="N15" s="130"/>
-      <c r="O15" s="40"/>
+      <c r="M15" s="167"/>
+      <c r="N15" s="168"/>
+      <c r="O15" s="171"/>
     </row>
     <row r="16" spans="1:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="4"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="136"/>
-      <c r="H16" s="137"/>
-      <c r="I16" s="139"/>
-      <c r="J16" s="83"/>
-      <c r="K16" s="84"/>
-      <c r="L16" s="86"/>
-      <c r="M16" s="131"/>
-      <c r="N16" s="132"/>
-      <c r="O16" s="41"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="49"/>
+      <c r="G16" s="52"/>
+      <c r="H16" s="53"/>
+      <c r="I16" s="55"/>
+      <c r="J16" s="58"/>
+      <c r="K16" s="59"/>
+      <c r="L16" s="61"/>
+      <c r="M16" s="169"/>
+      <c r="N16" s="170"/>
+      <c r="O16" s="172"/>
     </row>
     <row r="17" spans="2:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="173" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="27"/>
-      <c r="J17" s="27"/>
-      <c r="K17" s="27"/>
-      <c r="L17" s="27"/>
-      <c r="M17" s="27"/>
-      <c r="N17" s="27"/>
-      <c r="O17" s="28"/>
+      <c r="C17" s="174"/>
+      <c r="D17" s="174"/>
+      <c r="E17" s="174"/>
+      <c r="F17" s="174"/>
+      <c r="G17" s="174"/>
+      <c r="H17" s="174"/>
+      <c r="I17" s="174"/>
+      <c r="J17" s="174"/>
+      <c r="K17" s="174"/>
+      <c r="L17" s="174"/>
+      <c r="M17" s="174"/>
+      <c r="N17" s="174"/>
+      <c r="O17" s="175"/>
     </row>
     <row r="18" spans="2:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="29"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="30"/>
-      <c r="K18" s="30"/>
-      <c r="L18" s="30"/>
-      <c r="M18" s="30"/>
-      <c r="N18" s="30"/>
-      <c r="O18" s="31"/>
+      <c r="B18" s="176"/>
+      <c r="C18" s="177"/>
+      <c r="D18" s="177"/>
+      <c r="E18" s="177"/>
+      <c r="F18" s="177"/>
+      <c r="G18" s="177"/>
+      <c r="H18" s="177"/>
+      <c r="I18" s="177"/>
+      <c r="J18" s="177"/>
+      <c r="K18" s="177"/>
+      <c r="L18" s="177"/>
+      <c r="M18" s="177"/>
+      <c r="N18" s="177"/>
+      <c r="O18" s="178"/>
     </row>
     <row r="19" spans="2:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="32" t="s">
+      <c r="B19" s="179" t="s">
         <v>15</v>
       </c>
-      <c r="C19" s="33"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="104" t="s">
+      <c r="C19" s="180"/>
+      <c r="D19" s="180"/>
+      <c r="E19" s="180"/>
+      <c r="F19" s="180"/>
+      <c r="G19" s="96" t="s">
         <v>16</v>
       </c>
-      <c r="H19" s="105"/>
-      <c r="I19" s="106"/>
-      <c r="J19" s="75" t="s">
+      <c r="H19" s="97"/>
+      <c r="I19" s="98"/>
+      <c r="J19" s="102" t="s">
         <v>37</v>
       </c>
-      <c r="K19" s="76"/>
-      <c r="L19" s="77"/>
-      <c r="M19" s="133"/>
-      <c r="N19" s="93"/>
-      <c r="O19" s="94"/>
+      <c r="K19" s="103"/>
+      <c r="L19" s="104"/>
+      <c r="M19" s="187"/>
+      <c r="N19" s="108"/>
+      <c r="O19" s="109"/>
     </row>
     <row r="20" spans="2:15" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="32"/>
-      <c r="C20" s="33"/>
-      <c r="D20" s="33"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="174"/>
-      <c r="H20" s="175"/>
-      <c r="I20" s="176"/>
-      <c r="J20" s="177"/>
-      <c r="K20" s="178"/>
-      <c r="L20" s="179"/>
-      <c r="M20" s="180"/>
-      <c r="N20" s="181"/>
-      <c r="O20" s="182"/>
+      <c r="B20" s="179"/>
+      <c r="C20" s="180"/>
+      <c r="D20" s="180"/>
+      <c r="E20" s="180"/>
+      <c r="F20" s="180"/>
+      <c r="G20" s="181"/>
+      <c r="H20" s="182"/>
+      <c r="I20" s="183"/>
+      <c r="J20" s="184"/>
+      <c r="K20" s="185"/>
+      <c r="L20" s="186"/>
+      <c r="M20" s="188"/>
+      <c r="N20" s="189"/>
+      <c r="O20" s="190"/>
     </row>
     <row r="21" spans="2:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="186" t="s">
+      <c r="B21" s="80" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="171"/>
-      <c r="G21" s="141" t="s">
+      <c r="D21" s="82"/>
+      <c r="E21" s="82"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="72" t="s">
         <v>35</v>
       </c>
-      <c r="H21" s="143" t="s">
+      <c r="H21" s="74" t="s">
         <v>14</v>
       </c>
-      <c r="I21" s="144"/>
-      <c r="J21" s="69" t="s">
+      <c r="I21" s="75"/>
+      <c r="J21" s="78" t="s">
         <v>35</v>
       </c>
-      <c r="K21" s="71" t="s">
+      <c r="K21" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="L21" s="72"/>
-      <c r="M21" s="22"/>
-      <c r="N21" s="18"/>
-      <c r="O21" s="19"/>
+      <c r="L21" s="63"/>
+      <c r="M21" s="66"/>
+      <c r="N21" s="68"/>
+      <c r="O21" s="69"/>
     </row>
     <row r="22" spans="2:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="187"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="183"/>
-      <c r="G22" s="142"/>
-      <c r="H22" s="145"/>
-      <c r="I22" s="146"/>
-      <c r="J22" s="70"/>
-      <c r="K22" s="73"/>
-      <c r="L22" s="74"/>
-      <c r="M22" s="23"/>
-      <c r="N22" s="20"/>
-      <c r="O22" s="21"/>
+      <c r="B22" s="81"/>
+      <c r="C22" s="84"/>
+      <c r="D22" s="84"/>
+      <c r="E22" s="84"/>
+      <c r="F22" s="85"/>
+      <c r="G22" s="73"/>
+      <c r="H22" s="76"/>
+      <c r="I22" s="77"/>
+      <c r="J22" s="79"/>
+      <c r="K22" s="64"/>
+      <c r="L22" s="65"/>
+      <c r="M22" s="67"/>
+      <c r="N22" s="70"/>
+      <c r="O22" s="71"/>
     </row>
     <row r="23" spans="2:15" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="188">
+      <c r="B23" s="28">
         <v>0.38</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="184"/>
-      <c r="G23" s="97" t="s">
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="H23" s="140" t="s">
+      <c r="H23" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="100"/>
-      <c r="J23" s="58" t="s">
+      <c r="I23" s="25"/>
+      <c r="J23" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="K23" s="64" t="s">
+      <c r="K23" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="L23" s="61"/>
-      <c r="M23" s="10"/>
-      <c r="N23" s="6"/>
-      <c r="O23" s="7"/>
+      <c r="L23" s="17"/>
+      <c r="M23" s="20"/>
+      <c r="N23" s="37"/>
+      <c r="O23" s="11"/>
     </row>
     <row r="24" spans="2:15" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="189"/>
-      <c r="C24" s="12" t="s">
+      <c r="B24" s="29"/>
+      <c r="C24" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="185"/>
-      <c r="G24" s="98"/>
-      <c r="H24" s="101"/>
-      <c r="I24" s="102"/>
-      <c r="J24" s="59"/>
-      <c r="K24" s="62"/>
-      <c r="L24" s="63"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="8"/>
-      <c r="O24" s="9"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="23"/>
+      <c r="H24" s="26"/>
+      <c r="I24" s="27"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="18"/>
+      <c r="L24" s="19"/>
+      <c r="M24" s="21"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="13"/>
     </row>
     <row r="25" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="188">
+      <c r="B25" s="28">
         <v>0.56999999999999995</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="184"/>
-      <c r="G25" s="97" t="s">
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="H25" s="147" t="s">
+      <c r="H25" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="I25" s="148"/>
-      <c r="J25" s="58" t="s">
+      <c r="I25" s="39"/>
+      <c r="J25" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="K25" s="65" t="s">
+      <c r="K25" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="L25" s="66"/>
-      <c r="M25" s="10"/>
-      <c r="N25" s="14"/>
-      <c r="O25" s="15"/>
+      <c r="L25" s="43"/>
+      <c r="M25" s="20"/>
+      <c r="N25" s="31"/>
+      <c r="O25" s="32"/>
     </row>
     <row r="26" spans="2:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="190"/>
-      <c r="C26" s="12" t="s">
+      <c r="B26" s="30"/>
+      <c r="C26" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="185"/>
-      <c r="G26" s="98"/>
-      <c r="H26" s="149"/>
-      <c r="I26" s="150"/>
-      <c r="J26" s="59"/>
-      <c r="K26" s="67"/>
-      <c r="L26" s="68"/>
-      <c r="M26" s="11"/>
-      <c r="N26" s="16"/>
-      <c r="O26" s="17"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="23"/>
+      <c r="H26" s="40"/>
+      <c r="I26" s="41"/>
+      <c r="J26" s="15"/>
+      <c r="K26" s="44"/>
+      <c r="L26" s="45"/>
+      <c r="M26" s="21"/>
+      <c r="N26" s="33"/>
+      <c r="O26" s="34"/>
     </row>
     <row r="27" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="190"/>
-      <c r="C27" s="172" t="s">
+      <c r="B27" s="30"/>
+      <c r="C27" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="D27" s="172"/>
-      <c r="E27" s="172"/>
-      <c r="F27" s="173"/>
-      <c r="G27" s="97" t="s">
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="47"/>
+      <c r="G27" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="H27" s="140" t="s">
+      <c r="H27" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="I27" s="100"/>
-      <c r="J27" s="58" t="s">
+      <c r="I27" s="25"/>
+      <c r="J27" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="K27" s="64" t="s">
+      <c r="K27" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="L27" s="61"/>
-      <c r="M27" s="10"/>
-      <c r="N27" s="6"/>
-      <c r="O27" s="7"/>
+      <c r="L27" s="17"/>
+      <c r="M27" s="20"/>
+      <c r="N27" s="37"/>
+      <c r="O27" s="11"/>
     </row>
     <row r="28" spans="2:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="189"/>
-      <c r="C28" s="12" t="s">
+      <c r="B28" s="29"/>
+      <c r="C28" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="185"/>
-      <c r="G28" s="98"/>
-      <c r="H28" s="101"/>
-      <c r="I28" s="102"/>
-      <c r="J28" s="59"/>
-      <c r="K28" s="62"/>
-      <c r="L28" s="63"/>
-      <c r="M28" s="11"/>
-      <c r="N28" s="8"/>
-      <c r="O28" s="9"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="26"/>
+      <c r="I28" s="27"/>
+      <c r="J28" s="15"/>
+      <c r="K28" s="18"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="21"/>
+      <c r="N28" s="12"/>
+      <c r="O28" s="13"/>
     </row>
     <row r="29" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="188">
+      <c r="B29" s="28">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="C29" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="184"/>
-      <c r="G29" s="97" t="s">
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="H29" s="99" t="s">
+      <c r="H29" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="I29" s="100"/>
-      <c r="J29" s="58" t="s">
+      <c r="I29" s="25"/>
+      <c r="J29" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="K29" s="60" t="s">
+      <c r="K29" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="L29" s="61"/>
-      <c r="M29" s="10"/>
-      <c r="N29" s="103"/>
-      <c r="O29" s="7"/>
+      <c r="L29" s="17"/>
+      <c r="M29" s="20"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="11"/>
     </row>
     <row r="30" spans="2:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="189"/>
-      <c r="C30" s="12" t="s">
+      <c r="B30" s="29"/>
+      <c r="C30" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="185"/>
-      <c r="G30" s="98"/>
-      <c r="H30" s="101"/>
-      <c r="I30" s="102"/>
-      <c r="J30" s="59"/>
-      <c r="K30" s="62"/>
-      <c r="L30" s="63"/>
-      <c r="M30" s="11"/>
-      <c r="N30" s="8"/>
-      <c r="O30" s="9"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="27"/>
+      <c r="J30" s="15"/>
+      <c r="K30" s="18"/>
+      <c r="L30" s="19"/>
+      <c r="M30" s="21"/>
+      <c r="N30" s="12"/>
+      <c r="O30" s="13"/>
     </row>
     <row r="31" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="188"/>
-      <c r="C31" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="184"/>
-      <c r="G31" s="97"/>
-      <c r="H31" s="99"/>
-      <c r="I31" s="100"/>
-      <c r="J31" s="58"/>
-      <c r="K31" s="60"/>
-      <c r="L31" s="61"/>
-      <c r="M31" s="10"/>
-      <c r="N31" s="103"/>
-      <c r="O31" s="7"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="22"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="25"/>
+      <c r="J31" s="14"/>
+      <c r="K31" s="16"/>
+      <c r="L31" s="17"/>
+      <c r="M31" s="20"/>
+      <c r="N31" s="10"/>
+      <c r="O31" s="11"/>
     </row>
     <row r="32" spans="2:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="189"/>
-      <c r="C32" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="185"/>
-      <c r="G32" s="98"/>
-      <c r="H32" s="101"/>
-      <c r="I32" s="102"/>
-      <c r="J32" s="59"/>
-      <c r="K32" s="62"/>
-      <c r="L32" s="63"/>
-      <c r="M32" s="11"/>
-      <c r="N32" s="8"/>
-      <c r="O32" s="9"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="23"/>
+      <c r="H32" s="26"/>
+      <c r="I32" s="27"/>
+      <c r="J32" s="15"/>
+      <c r="K32" s="18"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="21"/>
+      <c r="N32" s="12"/>
+      <c r="O32" s="13"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2885,57 +2881,19 @@
     <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="84">
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="C31:F31"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="N29:O30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="K31:L32"/>
-    <mergeCell ref="M29:M30"/>
-    <mergeCell ref="G29:G30"/>
-    <mergeCell ref="H29:I30"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="K29:L30"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="B25:B28"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="C24:F24"/>
-    <mergeCell ref="C25:F25"/>
-    <mergeCell ref="N25:O26"/>
-    <mergeCell ref="G27:G28"/>
-    <mergeCell ref="H27:I28"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="K27:L28"/>
-    <mergeCell ref="M27:M28"/>
-    <mergeCell ref="N27:O28"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="H25:I26"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="K25:L26"/>
-    <mergeCell ref="M25:M26"/>
-    <mergeCell ref="C26:F26"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="E15:F16"/>
-    <mergeCell ref="G15:H16"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="J15:K16"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="K21:L22"/>
-    <mergeCell ref="M21:M22"/>
-    <mergeCell ref="N21:O22"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="H23:I24"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="K23:L24"/>
-    <mergeCell ref="M23:M24"/>
-    <mergeCell ref="N23:O24"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="H21:I22"/>
-    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="O13:O14"/>
+    <mergeCell ref="M15:N16"/>
+    <mergeCell ref="O15:O16"/>
+    <mergeCell ref="B17:O18"/>
+    <mergeCell ref="B19:F20"/>
+    <mergeCell ref="G19:I20"/>
+    <mergeCell ref="J19:L20"/>
+    <mergeCell ref="M19:O20"/>
+    <mergeCell ref="G13:H14"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="J13:K14"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="M13:N14"/>
     <mergeCell ref="B21:B22"/>
     <mergeCell ref="C21:F22"/>
     <mergeCell ref="B2:D3"/>
@@ -2951,24 +2909,62 @@
     <mergeCell ref="E4:O6"/>
     <mergeCell ref="G9:O10"/>
     <mergeCell ref="E9:F10"/>
+    <mergeCell ref="E13:F14"/>
+    <mergeCell ref="K21:L22"/>
+    <mergeCell ref="M21:M22"/>
+    <mergeCell ref="N21:O22"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="H23:I24"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="K23:L24"/>
+    <mergeCell ref="M23:M24"/>
+    <mergeCell ref="N23:O24"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:I22"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="E15:F16"/>
+    <mergeCell ref="G15:H16"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="J15:K16"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="N25:O26"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="H27:I28"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="K27:L28"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="N27:O28"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="H25:I26"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="K25:L26"/>
+    <mergeCell ref="M25:M26"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="N29:O30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="K31:L32"/>
+    <mergeCell ref="M29:M30"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="H29:I30"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="K29:L30"/>
     <mergeCell ref="G31:G32"/>
     <mergeCell ref="H31:I32"/>
     <mergeCell ref="M31:M32"/>
     <mergeCell ref="N31:O32"/>
-    <mergeCell ref="E13:F14"/>
-    <mergeCell ref="G13:H14"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="J13:K14"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="M13:N14"/>
-    <mergeCell ref="O13:O14"/>
-    <mergeCell ref="M15:N16"/>
-    <mergeCell ref="O15:O16"/>
-    <mergeCell ref="B17:O18"/>
-    <mergeCell ref="B19:F20"/>
-    <mergeCell ref="G19:I20"/>
-    <mergeCell ref="J19:L20"/>
-    <mergeCell ref="M19:O20"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.11811023622047245" right="0.11811023622047245" top="0.15748031496062992" bottom="0" header="0.19685039370078741" footer="0"/>

</xml_diff>